<commit_message>
2026-03-18 upload done from linux machine
</commit_message>
<xml_diff>
--- a/data_collection/category.xlsx
+++ b/data_collection/category.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="204">
   <si>
     <t>Category</t>
   </si>
@@ -521,6 +521,36 @@
   </si>
   <si>
     <t>개인 및 가정용품 수리업</t>
+  </si>
+  <si>
+    <t>우량기업부</t>
+  </si>
+  <si>
+    <t>nan</t>
+  </si>
+  <si>
+    <t>SPAC(소속부없음)</t>
+  </si>
+  <si>
+    <t>투자주의환기종목(소속부없음)</t>
+  </si>
+  <si>
+    <t>관리종목(소속부없음)</t>
+  </si>
+  <si>
+    <t>중견기업부</t>
+  </si>
+  <si>
+    <t>외국기업(소속부없음)</t>
+  </si>
+  <si>
+    <t>기술성장기업부</t>
+  </si>
+  <si>
+    <t>일반기업부</t>
+  </si>
+  <si>
+    <t>벤처기업부</t>
   </si>
   <si>
     <t>IT</t>
@@ -953,7 +983,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B168"/>
+  <dimension ref="A1:B178"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -969,7 +999,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -977,7 +1007,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -985,7 +1015,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -993,7 +1023,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1001,7 +1031,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1009,7 +1039,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1017,7 +1047,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1025,7 +1055,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1033,7 +1063,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1041,7 +1071,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1049,7 +1079,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -1057,7 +1087,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1065,7 +1095,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -1073,7 +1103,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -1081,7 +1111,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -1089,7 +1119,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -1097,7 +1127,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1105,7 +1135,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1113,7 +1143,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1121,7 +1151,7 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1129,7 +1159,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1137,7 +1167,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1145,7 +1175,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1153,7 +1183,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1161,7 +1191,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1169,7 +1199,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -1177,7 +1207,7 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -1185,7 +1215,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -1193,7 +1223,7 @@
         <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -1201,7 +1231,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -1209,7 +1239,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -1217,7 +1247,7 @@
         <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -1225,7 +1255,7 @@
         <v>34</v>
       </c>
       <c r="B34" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -1233,7 +1263,7 @@
         <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -1241,7 +1271,7 @@
         <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -1249,7 +1279,7 @@
         <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -1257,7 +1287,7 @@
         <v>38</v>
       </c>
       <c r="B38" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -1265,7 +1295,7 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -1273,7 +1303,7 @@
         <v>40</v>
       </c>
       <c r="B40" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -1281,7 +1311,7 @@
         <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -1289,7 +1319,7 @@
         <v>42</v>
       </c>
       <c r="B42" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -1297,7 +1327,7 @@
         <v>43</v>
       </c>
       <c r="B43" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -1305,7 +1335,7 @@
         <v>44</v>
       </c>
       <c r="B44" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -1313,7 +1343,7 @@
         <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -1321,7 +1351,7 @@
         <v>46</v>
       </c>
       <c r="B46" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -1329,7 +1359,7 @@
         <v>47</v>
       </c>
       <c r="B47" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -1337,7 +1367,7 @@
         <v>48</v>
       </c>
       <c r="B48" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -1345,7 +1375,7 @@
         <v>49</v>
       </c>
       <c r="B49" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -1353,7 +1383,7 @@
         <v>50</v>
       </c>
       <c r="B50" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -1361,7 +1391,7 @@
         <v>51</v>
       </c>
       <c r="B51" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -1369,7 +1399,7 @@
         <v>52</v>
       </c>
       <c r="B52" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -1377,7 +1407,7 @@
         <v>53</v>
       </c>
       <c r="B53" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -1385,7 +1415,7 @@
         <v>54</v>
       </c>
       <c r="B54" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1393,7 +1423,7 @@
         <v>55</v>
       </c>
       <c r="B55" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1401,7 +1431,7 @@
         <v>56</v>
       </c>
       <c r="B56" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1409,7 +1439,7 @@
         <v>57</v>
       </c>
       <c r="B57" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1417,7 +1447,7 @@
         <v>58</v>
       </c>
       <c r="B58" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1425,7 +1455,7 @@
         <v>59</v>
       </c>
       <c r="B59" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1433,7 +1463,7 @@
         <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1441,7 +1471,7 @@
         <v>61</v>
       </c>
       <c r="B61" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1449,7 +1479,7 @@
         <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -1457,7 +1487,7 @@
         <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -1465,7 +1495,7 @@
         <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -1473,7 +1503,7 @@
         <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -1481,7 +1511,7 @@
         <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -1489,7 +1519,7 @@
         <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -1497,7 +1527,7 @@
         <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -1505,7 +1535,7 @@
         <v>69</v>
       </c>
       <c r="B69" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -1513,7 +1543,7 @@
         <v>70</v>
       </c>
       <c r="B70" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -1521,7 +1551,7 @@
         <v>71</v>
       </c>
       <c r="B71" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -1529,7 +1559,7 @@
         <v>72</v>
       </c>
       <c r="B72" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -1537,7 +1567,7 @@
         <v>73</v>
       </c>
       <c r="B73" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -1545,7 +1575,7 @@
         <v>74</v>
       </c>
       <c r="B74" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -1553,7 +1583,7 @@
         <v>75</v>
       </c>
       <c r="B75" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -1561,7 +1591,7 @@
         <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1569,7 +1599,7 @@
         <v>77</v>
       </c>
       <c r="B77" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1577,7 +1607,7 @@
         <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1585,7 +1615,7 @@
         <v>79</v>
       </c>
       <c r="B79" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1593,7 +1623,7 @@
         <v>80</v>
       </c>
       <c r="B80" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1601,7 +1631,7 @@
         <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1609,7 +1639,7 @@
         <v>82</v>
       </c>
       <c r="B82" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1617,7 +1647,7 @@
         <v>83</v>
       </c>
       <c r="B83" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1625,7 +1655,7 @@
         <v>84</v>
       </c>
       <c r="B84" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1633,7 +1663,7 @@
         <v>85</v>
       </c>
       <c r="B85" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1641,7 +1671,7 @@
         <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1649,7 +1679,7 @@
         <v>87</v>
       </c>
       <c r="B87" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1657,7 +1687,7 @@
         <v>88</v>
       </c>
       <c r="B88" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1665,7 +1695,7 @@
         <v>89</v>
       </c>
       <c r="B89" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1673,7 +1703,7 @@
         <v>90</v>
       </c>
       <c r="B90" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1681,7 +1711,7 @@
         <v>91</v>
       </c>
       <c r="B91" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1689,7 +1719,7 @@
         <v>92</v>
       </c>
       <c r="B92" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1697,7 +1727,7 @@
         <v>93</v>
       </c>
       <c r="B93" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1705,7 +1735,7 @@
         <v>94</v>
       </c>
       <c r="B94" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1713,7 +1743,7 @@
         <v>95</v>
       </c>
       <c r="B95" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1721,7 +1751,7 @@
         <v>96</v>
       </c>
       <c r="B96" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1729,7 +1759,7 @@
         <v>97</v>
       </c>
       <c r="B97" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1737,7 +1767,7 @@
         <v>98</v>
       </c>
       <c r="B98" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1745,7 +1775,7 @@
         <v>99</v>
       </c>
       <c r="B99" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1753,7 +1783,7 @@
         <v>100</v>
       </c>
       <c r="B100" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1761,7 +1791,7 @@
         <v>101</v>
       </c>
       <c r="B101" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1769,7 +1799,7 @@
         <v>102</v>
       </c>
       <c r="B102" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1777,7 +1807,7 @@
         <v>103</v>
       </c>
       <c r="B103" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1785,7 +1815,7 @@
         <v>104</v>
       </c>
       <c r="B104" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1793,7 +1823,7 @@
         <v>105</v>
       </c>
       <c r="B105" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1801,7 +1831,7 @@
         <v>106</v>
       </c>
       <c r="B106" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1809,7 +1839,7 @@
         <v>107</v>
       </c>
       <c r="B107" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1817,7 +1847,7 @@
         <v>108</v>
       </c>
       <c r="B108" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1825,7 +1855,7 @@
         <v>109</v>
       </c>
       <c r="B109" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1833,7 +1863,7 @@
         <v>110</v>
       </c>
       <c r="B110" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1841,7 +1871,7 @@
         <v>111</v>
       </c>
       <c r="B111" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1849,7 +1879,7 @@
         <v>112</v>
       </c>
       <c r="B112" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1857,7 +1887,7 @@
         <v>113</v>
       </c>
       <c r="B113" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1865,7 +1895,7 @@
         <v>114</v>
       </c>
       <c r="B114" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1873,7 +1903,7 @@
         <v>115</v>
       </c>
       <c r="B115" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1881,7 +1911,7 @@
         <v>116</v>
       </c>
       <c r="B116" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1889,7 +1919,7 @@
         <v>117</v>
       </c>
       <c r="B117" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1897,7 +1927,7 @@
         <v>118</v>
       </c>
       <c r="B118" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1905,7 +1935,7 @@
         <v>119</v>
       </c>
       <c r="B119" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1913,7 +1943,7 @@
         <v>120</v>
       </c>
       <c r="B120" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="121" spans="1:2">
@@ -1921,7 +1951,7 @@
         <v>121</v>
       </c>
       <c r="B121" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="122" spans="1:2">
@@ -1929,7 +1959,7 @@
         <v>122</v>
       </c>
       <c r="B122" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="123" spans="1:2">
@@ -1937,7 +1967,7 @@
         <v>123</v>
       </c>
       <c r="B123" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="124" spans="1:2">
@@ -1945,7 +1975,7 @@
         <v>124</v>
       </c>
       <c r="B124" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="125" spans="1:2">
@@ -1953,7 +1983,7 @@
         <v>125</v>
       </c>
       <c r="B125" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="126" spans="1:2">
@@ -1961,7 +1991,7 @@
         <v>126</v>
       </c>
       <c r="B126" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="127" spans="1:2">
@@ -1969,7 +1999,7 @@
         <v>127</v>
       </c>
       <c r="B127" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="128" spans="1:2">
@@ -1977,7 +2007,7 @@
         <v>128</v>
       </c>
       <c r="B128" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="129" spans="1:2">
@@ -1985,7 +2015,7 @@
         <v>129</v>
       </c>
       <c r="B129" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="130" spans="1:2">
@@ -1993,7 +2023,7 @@
         <v>130</v>
       </c>
       <c r="B130" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="131" spans="1:2">
@@ -2001,7 +2031,7 @@
         <v>131</v>
       </c>
       <c r="B131" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="132" spans="1:2">
@@ -2009,7 +2039,7 @@
         <v>132</v>
       </c>
       <c r="B132" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="133" spans="1:2">
@@ -2017,7 +2047,7 @@
         <v>133</v>
       </c>
       <c r="B133" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="134" spans="1:2">
@@ -2025,7 +2055,7 @@
         <v>134</v>
       </c>
       <c r="B134" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="135" spans="1:2">
@@ -2033,7 +2063,7 @@
         <v>135</v>
       </c>
       <c r="B135" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="136" spans="1:2">
@@ -2041,7 +2071,7 @@
         <v>136</v>
       </c>
       <c r="B136" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="137" spans="1:2">
@@ -2049,7 +2079,7 @@
         <v>137</v>
       </c>
       <c r="B137" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="138" spans="1:2">
@@ -2057,7 +2087,7 @@
         <v>138</v>
       </c>
       <c r="B138" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="139" spans="1:2">
@@ -2065,7 +2095,7 @@
         <v>139</v>
       </c>
       <c r="B139" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="140" spans="1:2">
@@ -2073,7 +2103,7 @@
         <v>140</v>
       </c>
       <c r="B140" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="141" spans="1:2">
@@ -2081,7 +2111,7 @@
         <v>141</v>
       </c>
       <c r="B141" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="142" spans="1:2">
@@ -2089,7 +2119,7 @@
         <v>142</v>
       </c>
       <c r="B142" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="143" spans="1:2">
@@ -2097,7 +2127,7 @@
         <v>143</v>
       </c>
       <c r="B143" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="144" spans="1:2">
@@ -2105,7 +2135,7 @@
         <v>144</v>
       </c>
       <c r="B144" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="145" spans="1:2">
@@ -2113,7 +2143,7 @@
         <v>145</v>
       </c>
       <c r="B145" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="146" spans="1:2">
@@ -2121,7 +2151,7 @@
         <v>146</v>
       </c>
       <c r="B146" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="147" spans="1:2">
@@ -2129,7 +2159,7 @@
         <v>147</v>
       </c>
       <c r="B147" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="148" spans="1:2">
@@ -2137,7 +2167,7 @@
         <v>148</v>
       </c>
       <c r="B148" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="149" spans="1:2">
@@ -2145,7 +2175,7 @@
         <v>149</v>
       </c>
       <c r="B149" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="150" spans="1:2">
@@ -2153,7 +2183,7 @@
         <v>150</v>
       </c>
       <c r="B150" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="151" spans="1:2">
@@ -2161,7 +2191,7 @@
         <v>151</v>
       </c>
       <c r="B151" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="152" spans="1:2">
@@ -2169,7 +2199,7 @@
         <v>152</v>
       </c>
       <c r="B152" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="153" spans="1:2">
@@ -2177,7 +2207,7 @@
         <v>153</v>
       </c>
       <c r="B153" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="154" spans="1:2">
@@ -2185,7 +2215,7 @@
         <v>154</v>
       </c>
       <c r="B154" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="155" spans="1:2">
@@ -2193,7 +2223,7 @@
         <v>155</v>
       </c>
       <c r="B155" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="156" spans="1:2">
@@ -2201,7 +2231,7 @@
         <v>156</v>
       </c>
       <c r="B156" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="157" spans="1:2">
@@ -2209,7 +2239,7 @@
         <v>157</v>
       </c>
       <c r="B157" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="158" spans="1:2">
@@ -2217,7 +2247,7 @@
         <v>158</v>
       </c>
       <c r="B158" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="159" spans="1:2">
@@ -2225,7 +2255,7 @@
         <v>159</v>
       </c>
       <c r="B159" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="160" spans="1:2">
@@ -2233,7 +2263,7 @@
         <v>160</v>
       </c>
       <c r="B160" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="161" spans="1:2">
@@ -2241,7 +2271,7 @@
         <v>161</v>
       </c>
       <c r="B161" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="162" spans="1:2">
@@ -2249,7 +2279,7 @@
         <v>162</v>
       </c>
       <c r="B162" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="163" spans="1:2">
@@ -2257,7 +2287,7 @@
         <v>163</v>
       </c>
       <c r="B163" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="164" spans="1:2">
@@ -2265,7 +2295,7 @@
         <v>164</v>
       </c>
       <c r="B164" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
     </row>
     <row r="165" spans="1:2">
@@ -2273,7 +2303,7 @@
         <v>165</v>
       </c>
       <c r="B165" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="166" spans="1:2">
@@ -2281,7 +2311,7 @@
         <v>166</v>
       </c>
       <c r="B166" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="167" spans="1:2">
@@ -2289,7 +2319,7 @@
         <v>167</v>
       </c>
       <c r="B167" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="168" spans="1:2">
@@ -2297,7 +2327,87 @@
         <v>168</v>
       </c>
       <c r="B168" t="s">
-        <v>193</v>
+        <v>203</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B169" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B170" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B171" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B172" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B173" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B174" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B175" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B176" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B177" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B178" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-03-19 upload done from linux machine
</commit_message>
<xml_diff>
--- a/data_collection/category.xlsx
+++ b/data_collection/category.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="203">
   <si>
     <t>Category</t>
   </si>
@@ -524,9 +524,6 @@
   </si>
   <si>
     <t>우량기업부</t>
-  </si>
-  <si>
-    <t>nan</t>
   </si>
   <si>
     <t>SPAC(소속부없음)</t>
@@ -999,7 +996,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1007,7 +1004,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1015,7 +1012,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1023,7 +1020,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1031,7 +1028,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1039,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1047,7 +1044,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1055,7 +1052,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1063,7 +1060,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1071,7 +1068,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1079,7 +1076,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -1087,7 +1084,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1095,7 +1092,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -1103,7 +1100,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -1111,7 +1108,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -1119,7 +1116,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -1127,7 +1124,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1135,7 +1132,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1143,7 +1140,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -1151,7 +1148,7 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1159,7 +1156,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -1167,7 +1164,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -1175,7 +1172,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1183,7 +1180,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1191,7 +1188,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -1199,7 +1196,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -1207,7 +1204,7 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -1215,7 +1212,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -1223,7 +1220,7 @@
         <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -1231,7 +1228,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -1239,7 +1236,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -1247,7 +1244,7 @@
         <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -1255,7 +1252,7 @@
         <v>34</v>
       </c>
       <c r="B34" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -1263,7 +1260,7 @@
         <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -1271,7 +1268,7 @@
         <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -1279,7 +1276,7 @@
         <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -1287,7 +1284,7 @@
         <v>38</v>
       </c>
       <c r="B38" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -1295,7 +1292,7 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -1303,7 +1300,7 @@
         <v>40</v>
       </c>
       <c r="B40" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -1311,7 +1308,7 @@
         <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -1319,7 +1316,7 @@
         <v>42</v>
       </c>
       <c r="B42" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -1327,7 +1324,7 @@
         <v>43</v>
       </c>
       <c r="B43" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -1335,7 +1332,7 @@
         <v>44</v>
       </c>
       <c r="B44" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -1343,7 +1340,7 @@
         <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -1351,7 +1348,7 @@
         <v>46</v>
       </c>
       <c r="B46" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -1359,7 +1356,7 @@
         <v>47</v>
       </c>
       <c r="B47" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -1367,7 +1364,7 @@
         <v>48</v>
       </c>
       <c r="B48" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -1375,7 +1372,7 @@
         <v>49</v>
       </c>
       <c r="B49" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -1383,7 +1380,7 @@
         <v>50</v>
       </c>
       <c r="B50" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -1391,7 +1388,7 @@
         <v>51</v>
       </c>
       <c r="B51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -1399,7 +1396,7 @@
         <v>52</v>
       </c>
       <c r="B52" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -1407,7 +1404,7 @@
         <v>53</v>
       </c>
       <c r="B53" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -1415,7 +1412,7 @@
         <v>54</v>
       </c>
       <c r="B54" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1423,7 +1420,7 @@
         <v>55</v>
       </c>
       <c r="B55" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1431,7 +1428,7 @@
         <v>56</v>
       </c>
       <c r="B56" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1439,7 +1436,7 @@
         <v>57</v>
       </c>
       <c r="B57" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1447,7 +1444,7 @@
         <v>58</v>
       </c>
       <c r="B58" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1455,7 +1452,7 @@
         <v>59</v>
       </c>
       <c r="B59" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1463,7 +1460,7 @@
         <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1471,7 +1468,7 @@
         <v>61</v>
       </c>
       <c r="B61" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1479,7 +1476,7 @@
         <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -1487,7 +1484,7 @@
         <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -1495,7 +1492,7 @@
         <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -1503,7 +1500,7 @@
         <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -1511,7 +1508,7 @@
         <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -1519,7 +1516,7 @@
         <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -1527,7 +1524,7 @@
         <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -1535,7 +1532,7 @@
         <v>69</v>
       </c>
       <c r="B69" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -1543,7 +1540,7 @@
         <v>70</v>
       </c>
       <c r="B70" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -1551,7 +1548,7 @@
         <v>71</v>
       </c>
       <c r="B71" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -1559,7 +1556,7 @@
         <v>72</v>
       </c>
       <c r="B72" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -1567,7 +1564,7 @@
         <v>73</v>
       </c>
       <c r="B73" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -1575,7 +1572,7 @@
         <v>74</v>
       </c>
       <c r="B74" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -1583,7 +1580,7 @@
         <v>75</v>
       </c>
       <c r="B75" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -1591,7 +1588,7 @@
         <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1599,7 +1596,7 @@
         <v>77</v>
       </c>
       <c r="B77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1607,7 +1604,7 @@
         <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1615,7 +1612,7 @@
         <v>79</v>
       </c>
       <c r="B79" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1623,7 +1620,7 @@
         <v>80</v>
       </c>
       <c r="B80" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1631,7 +1628,7 @@
         <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1639,7 +1636,7 @@
         <v>82</v>
       </c>
       <c r="B82" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1647,7 +1644,7 @@
         <v>83</v>
       </c>
       <c r="B83" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1655,7 +1652,7 @@
         <v>84</v>
       </c>
       <c r="B84" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1663,7 +1660,7 @@
         <v>85</v>
       </c>
       <c r="B85" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1671,7 +1668,7 @@
         <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1679,7 +1676,7 @@
         <v>87</v>
       </c>
       <c r="B87" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1687,7 +1684,7 @@
         <v>88</v>
       </c>
       <c r="B88" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1695,7 +1692,7 @@
         <v>89</v>
       </c>
       <c r="B89" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1703,7 +1700,7 @@
         <v>90</v>
       </c>
       <c r="B90" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1711,7 +1708,7 @@
         <v>91</v>
       </c>
       <c r="B91" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1719,7 +1716,7 @@
         <v>92</v>
       </c>
       <c r="B92" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1727,7 +1724,7 @@
         <v>93</v>
       </c>
       <c r="B93" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1735,7 +1732,7 @@
         <v>94</v>
       </c>
       <c r="B94" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1743,7 +1740,7 @@
         <v>95</v>
       </c>
       <c r="B95" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1751,7 +1748,7 @@
         <v>96</v>
       </c>
       <c r="B96" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1759,7 +1756,7 @@
         <v>97</v>
       </c>
       <c r="B97" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1767,7 +1764,7 @@
         <v>98</v>
       </c>
       <c r="B98" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1775,7 +1772,7 @@
         <v>99</v>
       </c>
       <c r="B99" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1783,7 +1780,7 @@
         <v>100</v>
       </c>
       <c r="B100" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1791,7 +1788,7 @@
         <v>101</v>
       </c>
       <c r="B101" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1799,7 +1796,7 @@
         <v>102</v>
       </c>
       <c r="B102" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="103" spans="1:2">
@@ -1807,7 +1804,7 @@
         <v>103</v>
       </c>
       <c r="B103" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="104" spans="1:2">
@@ -1815,7 +1812,7 @@
         <v>104</v>
       </c>
       <c r="B104" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="105" spans="1:2">
@@ -1823,7 +1820,7 @@
         <v>105</v>
       </c>
       <c r="B105" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="106" spans="1:2">
@@ -1831,7 +1828,7 @@
         <v>106</v>
       </c>
       <c r="B106" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="107" spans="1:2">
@@ -1839,7 +1836,7 @@
         <v>107</v>
       </c>
       <c r="B107" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="108" spans="1:2">
@@ -1847,7 +1844,7 @@
         <v>108</v>
       </c>
       <c r="B108" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="109" spans="1:2">
@@ -1855,7 +1852,7 @@
         <v>109</v>
       </c>
       <c r="B109" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="110" spans="1:2">
@@ -1863,7 +1860,7 @@
         <v>110</v>
       </c>
       <c r="B110" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="111" spans="1:2">
@@ -1871,7 +1868,7 @@
         <v>111</v>
       </c>
       <c r="B111" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="112" spans="1:2">
@@ -1879,7 +1876,7 @@
         <v>112</v>
       </c>
       <c r="B112" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="113" spans="1:2">
@@ -1887,7 +1884,7 @@
         <v>113</v>
       </c>
       <c r="B113" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="114" spans="1:2">
@@ -1895,7 +1892,7 @@
         <v>114</v>
       </c>
       <c r="B114" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="115" spans="1:2">
@@ -1903,7 +1900,7 @@
         <v>115</v>
       </c>
       <c r="B115" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="116" spans="1:2">
@@ -1911,7 +1908,7 @@
         <v>116</v>
       </c>
       <c r="B116" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="117" spans="1:2">
@@ -1919,7 +1916,7 @@
         <v>117</v>
       </c>
       <c r="B117" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="118" spans="1:2">
@@ -1927,7 +1924,7 @@
         <v>118</v>
       </c>
       <c r="B118" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="119" spans="1:2">
@@ -1935,7 +1932,7 @@
         <v>119</v>
       </c>
       <c r="B119" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="120" spans="1:2">
@@ -1943,7 +1940,7 @@
         <v>120</v>
       </c>
       <c r="B120" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="121" spans="1:2">
@@ -1951,7 +1948,7 @@
         <v>121</v>
       </c>
       <c r="B121" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="122" spans="1:2">
@@ -1959,7 +1956,7 @@
         <v>122</v>
       </c>
       <c r="B122" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="123" spans="1:2">
@@ -1967,7 +1964,7 @@
         <v>123</v>
       </c>
       <c r="B123" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="124" spans="1:2">
@@ -1975,7 +1972,7 @@
         <v>124</v>
       </c>
       <c r="B124" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="125" spans="1:2">
@@ -1983,7 +1980,7 @@
         <v>125</v>
       </c>
       <c r="B125" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="126" spans="1:2">
@@ -1991,7 +1988,7 @@
         <v>126</v>
       </c>
       <c r="B126" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="127" spans="1:2">
@@ -1999,7 +1996,7 @@
         <v>127</v>
       </c>
       <c r="B127" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="128" spans="1:2">
@@ -2007,7 +2004,7 @@
         <v>128</v>
       </c>
       <c r="B128" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="129" spans="1:2">
@@ -2015,7 +2012,7 @@
         <v>129</v>
       </c>
       <c r="B129" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="130" spans="1:2">
@@ -2023,7 +2020,7 @@
         <v>130</v>
       </c>
       <c r="B130" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="131" spans="1:2">
@@ -2031,7 +2028,7 @@
         <v>131</v>
       </c>
       <c r="B131" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="132" spans="1:2">
@@ -2039,7 +2036,7 @@
         <v>132</v>
       </c>
       <c r="B132" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="133" spans="1:2">
@@ -2047,7 +2044,7 @@
         <v>133</v>
       </c>
       <c r="B133" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="134" spans="1:2">
@@ -2055,7 +2052,7 @@
         <v>134</v>
       </c>
       <c r="B134" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="135" spans="1:2">
@@ -2063,7 +2060,7 @@
         <v>135</v>
       </c>
       <c r="B135" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="136" spans="1:2">
@@ -2071,7 +2068,7 @@
         <v>136</v>
       </c>
       <c r="B136" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="137" spans="1:2">
@@ -2079,7 +2076,7 @@
         <v>137</v>
       </c>
       <c r="B137" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="138" spans="1:2">
@@ -2087,7 +2084,7 @@
         <v>138</v>
       </c>
       <c r="B138" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="139" spans="1:2">
@@ -2095,7 +2092,7 @@
         <v>139</v>
       </c>
       <c r="B139" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="140" spans="1:2">
@@ -2103,7 +2100,7 @@
         <v>140</v>
       </c>
       <c r="B140" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="141" spans="1:2">
@@ -2111,7 +2108,7 @@
         <v>141</v>
       </c>
       <c r="B141" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="142" spans="1:2">
@@ -2119,7 +2116,7 @@
         <v>142</v>
       </c>
       <c r="B142" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="143" spans="1:2">
@@ -2127,7 +2124,7 @@
         <v>143</v>
       </c>
       <c r="B143" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="144" spans="1:2">
@@ -2135,7 +2132,7 @@
         <v>144</v>
       </c>
       <c r="B144" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="145" spans="1:2">
@@ -2143,7 +2140,7 @@
         <v>145</v>
       </c>
       <c r="B145" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="146" spans="1:2">
@@ -2151,7 +2148,7 @@
         <v>146</v>
       </c>
       <c r="B146" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="147" spans="1:2">
@@ -2159,7 +2156,7 @@
         <v>147</v>
       </c>
       <c r="B147" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="148" spans="1:2">
@@ -2167,7 +2164,7 @@
         <v>148</v>
       </c>
       <c r="B148" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="149" spans="1:2">
@@ -2175,7 +2172,7 @@
         <v>149</v>
       </c>
       <c r="B149" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="150" spans="1:2">
@@ -2183,7 +2180,7 @@
         <v>150</v>
       </c>
       <c r="B150" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="151" spans="1:2">
@@ -2191,7 +2188,7 @@
         <v>151</v>
       </c>
       <c r="B151" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="152" spans="1:2">
@@ -2199,7 +2196,7 @@
         <v>152</v>
       </c>
       <c r="B152" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="153" spans="1:2">
@@ -2207,7 +2204,7 @@
         <v>153</v>
       </c>
       <c r="B153" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="154" spans="1:2">
@@ -2215,7 +2212,7 @@
         <v>154</v>
       </c>
       <c r="B154" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="155" spans="1:2">
@@ -2223,7 +2220,7 @@
         <v>155</v>
       </c>
       <c r="B155" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="156" spans="1:2">
@@ -2231,7 +2228,7 @@
         <v>156</v>
       </c>
       <c r="B156" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="157" spans="1:2">
@@ -2239,7 +2236,7 @@
         <v>157</v>
       </c>
       <c r="B157" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="158" spans="1:2">
@@ -2247,7 +2244,7 @@
         <v>158</v>
       </c>
       <c r="B158" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="159" spans="1:2">
@@ -2255,7 +2252,7 @@
         <v>159</v>
       </c>
       <c r="B159" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="160" spans="1:2">
@@ -2263,7 +2260,7 @@
         <v>160</v>
       </c>
       <c r="B160" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="161" spans="1:2">
@@ -2271,7 +2268,7 @@
         <v>161</v>
       </c>
       <c r="B161" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="162" spans="1:2">
@@ -2279,7 +2276,7 @@
         <v>162</v>
       </c>
       <c r="B162" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="163" spans="1:2">
@@ -2287,7 +2284,7 @@
         <v>163</v>
       </c>
       <c r="B163" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="164" spans="1:2">
@@ -2295,7 +2292,7 @@
         <v>164</v>
       </c>
       <c r="B164" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="165" spans="1:2">
@@ -2303,7 +2300,7 @@
         <v>165</v>
       </c>
       <c r="B165" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="166" spans="1:2">
@@ -2311,7 +2308,7 @@
         <v>166</v>
       </c>
       <c r="B166" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="167" spans="1:2">
@@ -2319,7 +2316,7 @@
         <v>167</v>
       </c>
       <c r="B167" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="168" spans="1:2">
@@ -2327,7 +2324,7 @@
         <v>168</v>
       </c>
       <c r="B168" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="169" spans="1:2">
@@ -2335,79 +2332,77 @@
         <v>169</v>
       </c>
       <c r="B169" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="170" spans="1:2">
-      <c r="A170" s="1" t="s">
-        <v>170</v>
-      </c>
+      <c r="A170" s="1"/>
       <c r="B170" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B171" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B172" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B173" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B174" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B175" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B176" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B177" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B178" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>